<commit_message>
Hold Indian Institute of Management Lucknow pages for QA revision
</commit_message>
<xml_diff>
--- a/data/college-content-master.xlsx
+++ b/data/college-content-master.xlsx
@@ -759,32 +759,32 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.iiml.ac.in</t>
+          <t>https://www.iiml.ac.in/</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Pending Audit</t>
+          <t>37</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Research Complete</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Skipped - existing pages protected</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Already Exists</t>
+          <t>Blocked - QA &lt;= 70 or critical failure</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Checked</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.iimv.ac.in/</t>
+          <t>https://www.iimv.ac.in</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">

</xml_diff>